<commit_message>
Correzione checklist ID 32 e 40
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDIANETSERVIZISRLX1/MedianetServizi/4Handy.it/2025.12/accreditamento-checklist_V8.2.7.xlsx
+++ b/GATEWAY/A1#111#MEDIANETSERVIZISRLX1/MedianetServizi/4Handy.it/2025.12/accreditamento-checklist_V8.2.7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\A1#111#MEDIANETSERVIZISRLX1\MedianetServizi\4Handy.it\2025.12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FAA8D2-90F3-4A3A-A62C-9B881E99B7F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB54EF0-F72D-4D0B-B540-A3D61EA29FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="326">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -3663,15 +3663,9 @@
       <c r="M11" s="35"/>
       <c r="N11" s="35"/>
       <c r="O11" s="35"/>
-      <c r="P11" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q11" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="R11" s="35" t="s">
-        <v>95</v>
-      </c>
+      <c r="P11" s="35"/>
+      <c r="Q11" s="35"/>
+      <c r="R11" s="35"/>
       <c r="S11" s="35"/>
       <c r="T11" s="35"/>
       <c r="U11" s="36"/>
@@ -3751,15 +3745,9 @@
       <c r="M13" s="35"/>
       <c r="N13" s="35"/>
       <c r="O13" s="35"/>
-      <c r="P13" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q13" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="R13" s="35" t="s">
-        <v>95</v>
-      </c>
+      <c r="P13" s="35"/>
+      <c r="Q13" s="35"/>
+      <c r="R13" s="35"/>
       <c r="S13" s="35"/>
       <c r="T13" s="35"/>
       <c r="U13" s="36"/>
@@ -12491,21 +12479,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -12649,32 +12622,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12692,6 +12655,31 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>